<commit_message>
Prepare Digital Patrol V2 on Laravel 13
</commit_message>
<xml_diff>
--- a/storage/template/TEMPLATE-JADWAL-PATROLI.xlsx
+++ b/storage/template/TEMPLATE-JADWAL-PATROLI.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11211"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/imamsyz/PhpstormProjects/digipatrol.id/storage/template/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CODE.ID\Muhammad Rizki Gajah\DigitalPatrol\digipatrol-backend\storage\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92C95726-3EAE-FD40-838B-C2023E050475}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2880" yWindow="2680" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2880" yWindow="2685" windowWidth="30240" windowHeight="18885" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="JADWAL PATROLI" sheetId="7" r:id="rId1"/>
@@ -139,7 +138,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="hh\:mm"/>
   </numFmts>
@@ -323,12 +322,12 @@
     </dxf>
   </dxfs>
   <tableStyles count="2">
-    <tableStyle name="SAMPLE KATEGORI-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+    <tableStyle name="SAMPLE KATEGORI-style" pivot="0" count="3">
       <tableStyleElement type="headerRow" dxfId="9"/>
       <tableStyleElement type="firstRowStripe" dxfId="8"/>
       <tableStyleElement type="secondRowStripe" dxfId="7"/>
     </tableStyle>
-    <tableStyle name="KATEGORI-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
+    <tableStyle name="KATEGORI-style" pivot="0" count="3">
       <tableStyleElement type="headerRow" dxfId="6"/>
       <tableStyleElement type="firstRowStripe" dxfId="5"/>
       <tableStyleElement type="secondRowStripe" dxfId="4"/>
@@ -542,15 +541,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DE28329-74F9-E246-A43B-03441B3463AD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A2:F37"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="4.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="10" t="s">
         <v>20</v>
       </c>
@@ -559,7 +558,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="10" t="s">
         <v>1</v>
       </c>
@@ -570,7 +569,7 @@
       <c r="D3" s="11"/>
       <c r="E3" s="11"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
         <v>2</v>
       </c>
@@ -580,7 +579,7 @@
       </c>
       <c r="D4" s="12"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
         <v>18</v>
       </c>
@@ -592,7 +591,7 @@
       <c r="E5" s="8"/>
       <c r="F5" s="3"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="9"/>
       <c r="B6" s="4">
         <v>1111</v>
@@ -607,7 +606,7 @@
         <v>4444</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="5">
         <v>1</v>
       </c>
@@ -624,7 +623,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="5">
         <v>2</v>
       </c>
@@ -641,7 +640,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="5">
         <v>3</v>
       </c>
@@ -658,7 +657,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="5">
         <v>4</v>
       </c>
@@ -675,7 +674,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="5">
         <v>5</v>
       </c>
@@ -692,7 +691,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="5">
         <v>6</v>
       </c>
@@ -709,7 +708,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="5">
         <v>7</v>
       </c>
@@ -726,7 +725,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="5">
         <v>8</v>
       </c>
@@ -743,7 +742,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="5">
         <v>9</v>
       </c>
@@ -760,7 +759,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="5">
         <v>10</v>
       </c>
@@ -777,7 +776,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="5">
         <v>11</v>
       </c>
@@ -794,7 +793,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="5">
         <v>12</v>
       </c>
@@ -811,7 +810,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="5">
         <v>13</v>
       </c>
@@ -828,7 +827,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="5">
         <v>14</v>
       </c>
@@ -845,7 +844,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="5">
         <v>15</v>
       </c>
@@ -862,7 +861,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="5">
         <v>16</v>
       </c>
@@ -879,7 +878,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="5">
         <v>17</v>
       </c>
@@ -896,7 +895,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="5">
         <v>18</v>
       </c>
@@ -913,7 +912,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="5">
         <v>19</v>
       </c>
@@ -930,7 +929,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="5">
         <v>20</v>
       </c>
@@ -947,7 +946,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="5">
         <v>21</v>
       </c>
@@ -964,7 +963,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" s="5">
         <v>22</v>
       </c>
@@ -981,7 +980,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" s="5">
         <v>23</v>
       </c>
@@ -998,7 +997,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" s="5">
         <v>24</v>
       </c>
@@ -1015,7 +1014,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" s="5">
         <v>25</v>
       </c>
@@ -1032,7 +1031,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" s="5">
         <v>26</v>
       </c>
@@ -1049,7 +1048,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" s="5">
         <v>27</v>
       </c>
@@ -1066,7 +1065,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" s="5">
         <v>28</v>
       </c>
@@ -1083,7 +1082,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" s="5">
         <v>29</v>
       </c>
@@ -1100,7 +1099,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" s="5">
         <v>30</v>
       </c>
@@ -1117,7 +1116,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B37" s="1"/>
     </row>
   </sheetData>
@@ -1148,19 +1147,19 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{946A24F4-F36E-6844-86C1-86981797E137}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>BULAN!$B$4:$B$11</xm:f>
           </x14:formula1>
           <xm:sqref>C4 E4:K4</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D9F50F0E-372F-3A45-94B9-4C2CBF669EEE}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>BULAN!$A$4:$A$15</xm:f>
           </x14:formula1>
           <xm:sqref>C3 F3:H3 J3:L3</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{167FC4DD-F93C-4444-96F3-052CEC1D2312}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>SHIFT!$B$3:$B$6</xm:f>
           </x14:formula1>
@@ -1173,14 +1172,14 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5427011B-65AD-4146-A0F9-4E95C526E51D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A2:E6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>25</v>
       </c>
@@ -1197,7 +1196,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -1214,7 +1213,7 @@
         <v>0.625</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -1231,7 +1230,7 @@
         <v>0.91666666666666663</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -1248,7 +1247,7 @@
         <v>0.29166666666666669</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -1271,14 +1270,14 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F7B8649-8753-2F41-9C37-96686A292ECD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A3:B15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -1286,7 +1285,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -1294,7 +1293,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -1302,7 +1301,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
@@ -1310,7 +1309,7 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -1318,7 +1317,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
@@ -1326,7 +1325,7 @@
         <v>2027</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
@@ -1334,7 +1333,7 @@
         <v>2028</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
@@ -1342,7 +1341,7 @@
         <v>2029</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>12</v>
       </c>
@@ -1350,22 +1349,22 @@
         <v>2030</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>16</v>
       </c>

</xml_diff>